<commit_message>
Apply the final check of the 400 labels: seven labels changed (change log with reasons), checked labels rebuilt from the sheet, validation and corrected ratio re-run
</commit_message>
<xml_diff>
--- a/checks/09-check-sheet.filled.xlsx
+++ b/checks/09-check-sheet.filled.xlsx
@@ -1473,13 +1473,17 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>N vs M: large empirical benchmark of 13 CI methods plus a concise unified review of them; not S/P either way, abstract does not settle how much is review</t>
+          <t>The paper does both jobs at scale: about 15 pages of unified review of existing methods and about 13 pages of new benchmark results. That clears the threshold easily. It is not a plain benchmark (N) because the review of existing methods is a stated co-contribution. Threshold used on all rows: new experiments count as 'substantial' only if they are a stated main contribution, get their own results section, are run by the authors over several tasks or datasets and produce new comparative findings</t>
         </is>
       </c>
     </row>
@@ -1893,13 +1897,13 @@
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>S vs M: calls itself a systematic review but also reports own simulation results and a comparison of 4 CI methods; abstract does not show how substantial the new work is</t>
+          <t>The main job is the review. The simulation is short and confirms known theory without new comparative findings, so it is not substantial. S.</t>
         </is>
       </c>
     </row>
@@ -6909,13 +6913,17 @@
       </c>
       <c r="J118" s="8" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="K118" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K118" s="8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L118" s="8" t="inlineStr">
         <is>
-          <t>P vs N: argues a framing (ACM) but also describes a reference implementation with benchmark results (LongMemEval 92%); tie-break 3 would make it N if the system is the main content, abstract does not settle</t>
+          <t>It argues a framing, then presents the authors' own system and evaluates it on two public benchmarks in a dedicated evaluation section. That matches rule 3 exactly. N, not P.</t>
         </is>
       </c>
     </row>
@@ -11090,13 +11098,17 @@
       </c>
       <c r="J74" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K74" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K74" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="L74" s="8" t="inlineStr">
         <is>
-          <t>Survey; its benchmarking of representative methods may be new (would push toward M), but review is the main job</t>
+          <t>The main job is a survey and taxonomy, but the authors also ran a new multi-task benchmark: a dedicated section of about 29% of the body, with new results. These are not numbers copied from the original papers. Under the threshold this is substantial, so M rather than S. This is the same standard that makes Core 13 M.</t>
         </is>
       </c>
     </row>
@@ -12914,13 +12926,13 @@
       </c>
       <c r="J109" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="K109" s="8" t="n"/>
       <c r="L109" s="8" t="inlineStr">
         <is>
-          <t>P vs N: philosophical essay on Labour/Capital plus a game-theoretic agent-based simulation with results; abstract does not settle which is the main content</t>
+          <t>This is a philosophical essay, but a central part is a new model and simulation whose results are in the abstract and are used as evidence ('The final confirming result of our analysis'). New results are a main content, so it is not P. It reviews no literature, so it is not S or M. N. Borderline with P.</t>
         </is>
       </c>
     </row>
@@ -13386,17 +13398,13 @@
       </c>
       <c r="J118" s="8" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K118" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K118" s="8" t="n"/>
       <c r="L118" s="8" t="inlineStr">
         <is>
-          <t>Short conceptual proposal of a design process, no results and no literature synthesis (tie-break 7); borderline</t>
+          <t>The paper's job is to introduce a design method and illustrate it with a usage scenario. It does not argue a position or review a field. Rule 7 covers conceptual or normative proposals. This is a procedural method proposal with a worked demonstration, so it fits N ('new method') better than P. Borderline P vs N.</t>
         </is>
       </c>
     </row>
@@ -13602,13 +13610,17 @@
       </c>
       <c r="J122" s="8" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K122" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K122" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="L122" s="8" t="inlineStr">
         <is>
-          <t>System/architecture paper (Pico-Cloud) with use cases and some results; N fits, borderline vision paper</t>
+          <t>This is a vision or concept paper for an architecture class: use cases, design considerations, deployment models, challenges and comparison tables. There is no implementation or evaluation of its own, so it is not an N system paper. It is not mainly a literature synthesis either, since related work and prior-work numbers only support the concept. Rule 7 gives P. Borderline; S would also count as positive under rule 8.</t>
         </is>
       </c>
     </row>
@@ -15322,13 +15334,17 @@
       </c>
       <c r="J155" s="8" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="K155" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K155" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="L155" s="8" t="inlineStr">
         <is>
-          <t>U vs P/N: background review plus a proposed solution with no results (reads like a project proposal); abstract is clear enough that U may not fit, but P vs N not settled</t>
+          <t>The full text resolves the uncertainty, so U is wrong. The largest part is a review of existing detection work. The proposed architecture is conceptual, has no results and is presented as 'a technical guide'. That makes it a challenges-and-opportunities review with a roadmap. S (P would also be acceptable under rule 8). Not N or M, because there are no new experiments.</t>
         </is>
       </c>
     </row>
@@ -16370,13 +16386,17 @@
       </c>
       <c r="J175" s="8" t="inlineStr">
         <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="K175" s="8" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K175" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="L175" s="8" t="inlineStr">
         <is>
-          <t>N vs S: design space derived from analysis of existing kits and paper-interaction research, plus own kit designs; unclear whether the taxonomy of existing work or the new kits is the main contribution</t>
+          <t>The main contribution is a design space (taxonomy) synthesised from a structured review of existing kits and research, about two-thirds of the body. The authors' kits are short illustrative examples with no formal evaluation, so they are not a 'new system with evaluation' (M), and the review is not mere motivation (rule 2). S by main job. Borderline, because HCI design-space papers are often treated as N, but under this codebook a taxonomy built from the literature is S.</t>
         </is>
       </c>
     </row>
@@ -18410,13 +18430,13 @@
       </c>
       <c r="J214" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="K214" s="8" t="n"/>
       <c r="L214" s="8" t="inlineStr">
         <is>
-          <t>S vs M: survey that also reports own Monte Carlo simulations of attacks; abstract does not show how substantial the new experiments are</t>
+          <t>This is a survey with a small illustrative simulation. The simulation is not a main results section and is far below the size threshold. S.</t>
         </is>
       </c>
     </row>
@@ -19510,13 +19530,13 @@
       </c>
       <c r="J235" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="K235" s="8" t="n"/>
       <c r="L235" s="8" t="inlineStr">
         <is>
-          <t>S vs M: tutorial/review that also derives guarantees and runs a comprehensive simulation study comparing methods; abstract does not settle whether the new experiments are substantial</t>
+          <t>This is a tutorial or review. The simulation is the authors' own and has a results subsection, but it is small (about 16% of the body), uses toy synthetic processes only and serves to illustrate the reviewed methods. It is not a co-equal benchmark like Core 13 or Extra 73. S, borderline toward M.</t>
         </is>
       </c>
     </row>

</xml_diff>